<commit_message>
LDAP configurations included Slurm configurations accounting for VMs Hosts with virtual machines site.yml accounting for all the hosts now Renamed common to pre_ohpc
</commit_message>
<xml_diff>
--- a/roles/setup_slurm/files/slurm_conf.xlsx
+++ b/roles/setup_slurm/files/slurm_conf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jsequeira\vs_projects\ansible-puli\roles\setup-slurm\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jsequeira\vs_projects\ansible-puli\roles\setup_slurm\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AF8299-72AD-4533-80F4-5332C380EA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F413F33-2D18-43BC-B7B0-59C831350A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{787EF645-FDEF-D749-B29A-8997BAA1BD7D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{787EF645-FDEF-D749-B29A-8997BAA1BD7D}"/>
   </bookViews>
   <sheets>
     <sheet name="code" sheetId="4" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="645">
   <si>
     <t>Parameter</t>
   </si>
@@ -689,9 +689,6 @@
   </si>
   <si>
     <t>mps=cuda+RT+tensor=10752+336+84=11172 maximum number of processes that can be run on the GPU; decided to do sharding instead, see https://groups.google.com/g/slurm-users/c/3axnt5Wshkg and https://slurm.schedmd.com/gres.html#Sharding -&gt; 11172*2=22344</t>
-  </si>
-  <si>
-    <t>Will not have backup for now</t>
   </si>
   <si>
     <t xml:space="preserve">I think this will not be necessary if using the default slurmdbd. </t>
@@ -1833,21 +1830,6 @@
     <t>disable_send_gids</t>
   </si>
   <si>
-    <t>cpu[01-11] CPUs=32 Sockets=2 CoresPerSocket=16 ThreadsPerCore=2 RealMemory=128000 CpuBind=core</t>
-  </si>
-  <si>
-    <t>mem02 CPUs=32 Sockets=4 CoresPerSocket=16 ThreadsPerCore=2 RealMemory=1024000 Features=highmem CpuBind=core</t>
-  </si>
-  <si>
-    <t>highmem Nodes=mem02 MaxTime=10-00:00:00 AllowAccounts=MEM CpuBind=core DefMemPerCPU=42777</t>
-  </si>
-  <si>
-    <t>gpu Nodes=gpu[01-02] MaxTime=10-00:00:00 AllowAccounts=GPU AllowGroups=LAMSA CpuBind=core DefMemPerCPU=5333</t>
-  </si>
-  <si>
-    <t>cpu Nodes=cpu[01-11] MaxTime=30-00:00:00 AllowAccounts=CPU CpuBind=core DefMemPerCPU=5333 Default=YES</t>
-  </si>
-  <si>
     <t>AllowNoDefAcct</t>
   </si>
   <si>
@@ -2025,9 +2007,6 @@
     <t>By default, same value as DbdHost (i.e., mem1).</t>
   </si>
   <si>
-    <t>Will not specify one for now.</t>
-  </si>
-  <si>
     <t>Default is 6819.</t>
   </si>
   <si>
@@ -2100,9 +2079,6 @@
     <t>Suggested to not use "root" (the default).</t>
   </si>
   <si>
-    <t>For now won't backup the StorageHost. Must change this in the future.</t>
-  </si>
-  <si>
     <t>slurm_acct_db</t>
   </si>
   <si>
@@ -2130,13 +2106,7 @@
     <t>Same as the SlurmUser, if no problems arise.</t>
   </si>
   <si>
-    <t>Implements removal of mounted folders (including in container environment).</t>
-  </si>
-  <si>
     <t>/etc/slurm/epilog.sh</t>
-  </si>
-  <si>
-    <t>/etc/slurm/node_health_check.py</t>
   </si>
   <si>
     <t>Include temperature on the script.</t>
@@ -2169,12 +2139,6 @@
     </r>
   </si>
   <si>
-    <t>/etc/slurm/prolog.sh</t>
-  </si>
-  <si>
-    <t>Implements mounting of HOME and SCRATCH folders.</t>
-  </si>
-  <si>
     <t>Not relevant, a value of 0 prevents kernel from swapping out program data, value of 100 gives equal priority to swapping out file cache or anonymous pages. Also, this parameter is ignored now: https://slurm.schedmd.com/cgroup_v2.html#ignored_params</t>
   </si>
   <si>
@@ -2206,9 +2170,6 @@
     <t>gpu,shard</t>
   </si>
   <si>
-    <t>gpu[01-02] CPUs=32 Sockets=2 CoresPerSocket=16 ThreadsPerCore=2 RealMemory=128000 Features=nvidia Gres=gpu:nvidia:2,gpu:2,shard:22344 CpuBind=core</t>
-  </si>
-  <si>
     <t>SwitchName</t>
   </si>
   <si>
@@ -2234,6 +2195,45 @@
   </si>
   <si>
     <t>{{ bmc_password }}</t>
+  </si>
+  <si>
+    <t>/usr/sbin/nhc</t>
+  </si>
+  <si>
+    <t>Nothing for now.</t>
+  </si>
+  <si>
+    <t>Implements removal of processes for users with jobs no longer on the cluster (except for root).</t>
+  </si>
+  <si>
+    <t>slurmdbd1</t>
+  </si>
+  <si>
+    <t>slurmdbd2</t>
+  </si>
+  <si>
+    <t>slurmctld1</t>
+  </si>
+  <si>
+    <t>slurmctld2</t>
+  </si>
+  <si>
+    <t>scc-cpu[02-11]-10G CPUs=32 Sockets=2 CoresPerSocket=16 ThreadsPerCore=2 RealMemory=128000 CpuBind=core</t>
+  </si>
+  <si>
+    <t>scc-mem[01-2]-10G CPUs=32 Sockets=4 CoresPerSocket=16 ThreadsPerCore=2 RealMemory=1024000 Features=highmem CpuBind=core</t>
+  </si>
+  <si>
+    <t>scc-gpu[01-02]-10G CPUs=32 Sockets=2 CoresPerSocket=16 ThreadsPerCore=2 RealMemory=128000 Features=nvidia Gres=gpu:nvidia:2,gpu:2,shard:22344 CpuBind=core</t>
+  </si>
+  <si>
+    <t>cpu Nodes=scc-cpu[02-11]-10G MaxTime=30-00:00:00 AllowAccounts=CPU CpuBind=core DefMemPerCPU=5333 Default=YES</t>
+  </si>
+  <si>
+    <t>highmem Nodes=scc-mem[01-02]-10G MaxTime=10-00:00:00 AllowAccounts=MEM CpuBind=core DefMemPerCPU=42777</t>
+  </si>
+  <si>
+    <t>gpu Nodes=scc-gpu[01-02]-10G MaxTime=10-00:00:00 AllowAccounts=GPU AllowGroups=LAMSA CpuBind=core DefMemPerCPU=5333</t>
   </si>
 </sst>
 </file>
@@ -2454,7 +2454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2558,6 +2558,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2931,8 +2934,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{51CC044A-B762-644D-ACB7-A7A2D791F53F}" name="Tabela1" displayName="Tabela1" ref="A1:C217" totalsRowShown="0" dataDxfId="51">
-  <autoFilter ref="A1:C217" xr:uid="{51CC044A-B762-644D-ACB7-A7A2D791F53F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{51CC044A-B762-644D-ACB7-A7A2D791F53F}" name="Tabela1" displayName="Tabela1" ref="A1:C218" totalsRowShown="0" dataDxfId="51">
+  <autoFilter ref="A1:C218" xr:uid="{51CC044A-B762-644D-ACB7-A7A2D791F53F}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{6D9AE7F7-3B19-3746-9C10-9B5E5D9E77F7}" name="Parameter" dataDxfId="50"/>
     <tableColumn id="2" xr3:uid="{7647DEBD-2263-2948-B456-6D4BB0FFCC72}" name="Value" dataDxfId="49"/>
@@ -3355,32 +3358,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -3411,98 +3414,98 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -3538,7 +3541,7 @@
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="17" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3556,7 +3559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6E252AF-4204-7C46-A81A-FB82CF0AB19E}">
-  <dimension ref="A1:C217"/>
+  <dimension ref="A1:C218"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.625" customWidth="1"/>
@@ -3579,10 +3582,10 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="6" t="s">
-        <v>215</v>
-      </c>
+      <c r="B2" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="C2" s="6"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3592,7 +3595,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3601,7 +3604,7 @@
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3609,7 +3612,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -3619,7 +3622,7 @@
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3627,10 +3630,10 @@
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>218</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3641,7 +3644,7 @@
         <v>6819</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3649,10 +3652,10 @@
         <v>11</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>221</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3660,10 +3663,10 @@
         <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3671,10 +3674,10 @@
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>640</v>
+        <v>627</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>620</v>
+        <v>612</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3682,10 +3685,10 @@
         <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>233</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3696,7 +3699,7 @@
         <v>300</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3704,10 +3707,10 @@
         <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3716,7 +3719,7 @@
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -3725,7 +3728,7 @@
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3733,10 +3736,10 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3744,10 +3747,10 @@
         <v>20</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -3756,7 +3759,7 @@
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -3765,7 +3768,7 @@
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -3774,7 +3777,7 @@
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -3785,7 +3788,7 @@
         <v>210</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -3794,7 +3797,7 @@
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -3803,7 +3806,7 @@
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3812,7 +3815,7 @@
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3821,7 +3824,7 @@
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -3830,7 +3833,7 @@
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -3838,10 +3841,10 @@
         <v>30</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -3850,7 +3853,7 @@
       </c>
       <c r="B29" s="1"/>
       <c r="C29" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -3858,7 +3861,7 @@
         <v>32</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>641</v>
+        <v>628</v>
       </c>
       <c r="C30" s="6"/>
     </row>
@@ -3875,7 +3878,7 @@
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -3884,7 +3887,7 @@
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -3893,7 +3896,7 @@
       </c>
       <c r="B34" s="1"/>
       <c r="C34" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -3902,7 +3905,7 @@
       </c>
       <c r="B35" s="1"/>
       <c r="C35" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -3911,7 +3914,7 @@
       </c>
       <c r="B36" s="1"/>
       <c r="C36" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -3920,7 +3923,7 @@
       </c>
       <c r="B37" s="1"/>
       <c r="C37" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3929,7 +3932,7 @@
       </c>
       <c r="B38" s="1"/>
       <c r="C38" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -3938,7 +3941,7 @@
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -3947,7 +3950,7 @@
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -3959,7 +3962,7 @@
         <v>5120</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -3968,7 +3971,7 @@
       </c>
       <c r="B42" s="1"/>
       <c r="C42" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -3977,7 +3980,7 @@
       </c>
       <c r="B43" s="1"/>
       <c r="C43" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -3986,7 +3989,7 @@
       </c>
       <c r="B44" s="1"/>
       <c r="C44" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -3995,7 +3998,7 @@
       </c>
       <c r="B45" s="1"/>
       <c r="C45" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -4004,7 +4007,7 @@
       </c>
       <c r="B46" s="1"/>
       <c r="C46" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -4012,10 +4015,10 @@
         <v>49</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>279</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -4023,10 +4026,10 @@
         <v>50</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>622</v>
+        <v>613</v>
       </c>
       <c r="C48" s="36" t="s">
-        <v>621</v>
+        <v>634</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -4035,7 +4038,7 @@
       </c>
       <c r="B49" s="1"/>
       <c r="C49" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -4044,7 +4047,7 @@
       </c>
       <c r="B50" s="1"/>
       <c r="C50" s="10" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -4055,7 +4058,7 @@
         <v>5</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -4064,7 +4067,7 @@
       </c>
       <c r="B52" s="1"/>
       <c r="C52" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -4073,7 +4076,7 @@
       </c>
       <c r="B53" s="1"/>
       <c r="C53" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -4082,7 +4085,7 @@
       </c>
       <c r="B54" s="1"/>
       <c r="C54" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -4090,10 +4093,10 @@
         <v>57</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>634</v>
+        <v>622</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -4102,7 +4105,7 @@
       </c>
       <c r="B56" s="1"/>
       <c r="C56" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -4111,7 +4114,7 @@
       </c>
       <c r="B57" s="1"/>
       <c r="C57" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -4119,10 +4122,10 @@
         <v>60</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -4131,7 +4134,7 @@
       </c>
       <c r="B59" s="1"/>
       <c r="C59" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -4142,7 +4145,7 @@
         <v>300</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -4150,10 +4153,10 @@
         <v>63</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -4161,10 +4164,10 @@
         <v>64</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>623</v>
+        <v>632</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>624</v>
+        <v>614</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -4172,10 +4175,10 @@
         <v>65</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -4184,7 +4187,7 @@
       </c>
       <c r="B64" s="1"/>
       <c r="C64" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -4192,7 +4195,7 @@
         <v>67</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C65" s="3"/>
     </row>
@@ -4201,10 +4204,10 @@
         <v>68</v>
       </c>
       <c r="B66" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="C66" s="6" t="s">
         <v>297</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4213,7 +4216,7 @@
       </c>
       <c r="B67" s="1"/>
       <c r="C67" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -4221,7 +4224,7 @@
         <v>70</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>639</v>
+        <v>626</v>
       </c>
       <c r="C68" s="3"/>
     </row>
@@ -4230,10 +4233,10 @@
         <v>71</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C69" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -4242,7 +4245,7 @@
       </c>
       <c r="B70" s="1"/>
       <c r="C70" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -4250,7 +4253,7 @@
         <v>73</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C71" s="4"/>
     </row>
@@ -4268,7 +4271,7 @@
         <v>75</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C73" s="3"/>
     </row>
@@ -4277,7 +4280,7 @@
         <v>76</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>625</v>
+        <v>615</v>
       </c>
       <c r="C74" s="4"/>
     </row>
@@ -4286,10 +4289,10 @@
         <v>77</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>619</v>
+        <v>611</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -4298,7 +4301,7 @@
       </c>
       <c r="B76" s="1"/>
       <c r="C76" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -4307,7 +4310,7 @@
       </c>
       <c r="B77" s="1"/>
       <c r="C77" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
@@ -4315,10 +4318,10 @@
         <v>80</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -4329,7 +4332,7 @@
         <v>1</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -4338,7 +4341,7 @@
       </c>
       <c r="B80" s="1"/>
       <c r="C80" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -4347,7 +4350,7 @@
       </c>
       <c r="B81" s="1"/>
       <c r="C81" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -4356,7 +4359,7 @@
       </c>
       <c r="B82" s="1"/>
       <c r="C82" s="10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4364,10 +4367,10 @@
         <v>85</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C83" s="33" t="s">
-        <v>626</v>
+        <v>616</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -4376,7 +4379,7 @@
       </c>
       <c r="B84" s="1"/>
       <c r="C84" s="10" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -4385,7 +4388,7 @@
       </c>
       <c r="B85" s="1"/>
       <c r="C85" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -4394,7 +4397,7 @@
       </c>
       <c r="B86" s="1"/>
       <c r="C86" s="6" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -4403,7 +4406,7 @@
       </c>
       <c r="B87" s="1"/>
       <c r="C87" s="6" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -4412,7 +4415,7 @@
       </c>
       <c r="B88" s="1"/>
       <c r="C88" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -4421,7 +4424,7 @@
       </c>
       <c r="B89" s="1"/>
       <c r="C89" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -4430,7 +4433,7 @@
       </c>
       <c r="B90" s="1"/>
       <c r="C90" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -4439,7 +4442,7 @@
       </c>
       <c r="B91" s="1"/>
       <c r="C91" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -4448,7 +4451,7 @@
       </c>
       <c r="B92" s="1"/>
       <c r="C92" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -4457,7 +4460,7 @@
       </c>
       <c r="B93" s="1"/>
       <c r="C93" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -4468,7 +4471,7 @@
         <v>11</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -4477,7 +4480,7 @@
       </c>
       <c r="B95" s="1"/>
       <c r="C95" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -4486,7 +4489,7 @@
       </c>
       <c r="B96" s="1"/>
       <c r="C96" s="3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4495,7 +4498,7 @@
       </c>
       <c r="B97" s="1"/>
       <c r="C97" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="63" x14ac:dyDescent="0.25">
@@ -4504,7 +4507,7 @@
       </c>
       <c r="B98" s="1"/>
       <c r="C98" s="6" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4513,7 +4516,7 @@
       </c>
       <c r="B99" s="1"/>
       <c r="C99" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -4522,7 +4525,7 @@
       </c>
       <c r="B100" s="1"/>
       <c r="C100" s="3" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
@@ -4530,10 +4533,10 @@
         <v>103</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -4542,7 +4545,7 @@
       </c>
       <c r="B102" s="1"/>
       <c r="C102" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -4551,7 +4554,7 @@
       </c>
       <c r="B103" s="1"/>
       <c r="C103" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -4560,7 +4563,7 @@
       </c>
       <c r="B104" s="1"/>
       <c r="C104" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -4569,7 +4572,7 @@
       </c>
       <c r="B105" s="1"/>
       <c r="C105" s="6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -4578,7 +4581,7 @@
       </c>
       <c r="B106" s="1"/>
       <c r="C106" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -4587,7 +4590,7 @@
       </c>
       <c r="B107" s="1"/>
       <c r="C107" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -4596,7 +4599,7 @@
       </c>
       <c r="B108" s="1"/>
       <c r="C108" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -4605,7 +4608,7 @@
       </c>
       <c r="B109" s="1"/>
       <c r="C109" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -4614,7 +4617,7 @@
       </c>
       <c r="B110" s="1"/>
       <c r="C110" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -4623,7 +4626,7 @@
       </c>
       <c r="B111" s="1"/>
       <c r="C111" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -4632,7 +4635,7 @@
       </c>
       <c r="B112" s="1"/>
       <c r="C112" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
@@ -4640,10 +4643,10 @@
         <v>115</v>
       </c>
       <c r="B113" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C113" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
@@ -4652,7 +4655,7 @@
       </c>
       <c r="B114" s="1"/>
       <c r="C114" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
@@ -4661,7 +4664,7 @@
       </c>
       <c r="B115" s="1"/>
       <c r="C115" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
@@ -4670,7 +4673,7 @@
       </c>
       <c r="B116" s="1"/>
       <c r="C116" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
@@ -4679,7 +4682,7 @@
       </c>
       <c r="B117" s="1"/>
       <c r="C117" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
@@ -4688,7 +4691,7 @@
       </c>
       <c r="B118" s="1"/>
       <c r="C118" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
@@ -4697,7 +4700,7 @@
       </c>
       <c r="B119" s="1"/>
       <c r="C119" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -4705,10 +4708,10 @@
         <v>122</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
@@ -4717,7 +4720,7 @@
       </c>
       <c r="B121" s="1"/>
       <c r="C121" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -4728,7 +4731,7 @@
         <v>1</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -4737,7 +4740,7 @@
       </c>
       <c r="B123" s="1"/>
       <c r="C123" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -4748,7 +4751,7 @@
         <v>1</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4757,7 +4760,7 @@
       </c>
       <c r="B125" s="1"/>
       <c r="C125" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
@@ -4766,7 +4769,7 @@
       </c>
       <c r="B126" s="1"/>
       <c r="C126" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
@@ -4775,7 +4778,7 @@
       </c>
       <c r="B127" s="1"/>
       <c r="C127" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4784,7 +4787,7 @@
       </c>
       <c r="B128" s="1"/>
       <c r="C128" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
@@ -4792,10 +4795,10 @@
         <v>131</v>
       </c>
       <c r="B129" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="C129" s="3" t="s">
         <v>434</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="130" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
@@ -4803,21 +4806,19 @@
         <v>132</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>630</v>
+        <v>618</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B131" s="1" t="s">
-        <v>627</v>
-      </c>
-      <c r="C131" s="36" t="s">
-        <v>628</v>
+      <c r="B131" s="1"/>
+      <c r="C131" s="38" t="s">
+        <v>633</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -4826,7 +4827,7 @@
       </c>
       <c r="B132" s="1"/>
       <c r="C132" s="10" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -4834,10 +4835,10 @@
         <v>135</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -4846,7 +4847,7 @@
       </c>
       <c r="B134" s="1"/>
       <c r="C134" s="10" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="135" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4855,7 +4856,7 @@
       </c>
       <c r="B135" s="1"/>
       <c r="C135" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -4864,7 +4865,7 @@
       </c>
       <c r="B136" s="1"/>
       <c r="C136" s="3" t="s">
-        <v>631</v>
+        <v>619</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -4873,7 +4874,7 @@
       </c>
       <c r="B137" s="1"/>
       <c r="C137" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -4882,7 +4883,7 @@
       </c>
       <c r="B138" s="1"/>
       <c r="C138" s="10" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="139" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4891,7 +4892,7 @@
       </c>
       <c r="B139" s="1"/>
       <c r="C139" s="10" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="140" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4900,7 +4901,7 @@
       </c>
       <c r="B140" s="1"/>
       <c r="C140" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
@@ -4909,7 +4910,7 @@
       </c>
       <c r="B141" s="1"/>
       <c r="C141" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="142" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4918,7 +4919,7 @@
       </c>
       <c r="B142" s="1"/>
       <c r="C142" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="143" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4927,7 +4928,7 @@
       </c>
       <c r="B143" s="1"/>
       <c r="C143" s="10" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -4936,7 +4937,7 @@
       </c>
       <c r="B144" s="1"/>
       <c r="C144" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="145" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4945,7 +4946,7 @@
       </c>
       <c r="B145" s="1"/>
       <c r="C145" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="146" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4954,7 +4955,7 @@
       </c>
       <c r="B146" s="1"/>
       <c r="C146" s="10" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
@@ -4963,7 +4964,7 @@
       </c>
       <c r="B147" s="1"/>
       <c r="C147" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
@@ -4972,7 +4973,7 @@
       </c>
       <c r="B148" s="1"/>
       <c r="C148" s="3" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="149" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -4981,7 +4982,7 @@
       </c>
       <c r="B149" s="1"/>
       <c r="C149" s="3" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="150" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
@@ -4989,10 +4990,10 @@
         <v>152</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C150" s="10" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -5001,7 +5002,7 @@
       </c>
       <c r="B151" s="1"/>
       <c r="C151" s="3" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
@@ -5012,7 +5013,7 @@
         <v>211</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="153" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -5020,10 +5021,10 @@
         <v>155</v>
       </c>
       <c r="B153" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C153" s="3" t="s">
         <v>456</v>
-      </c>
-      <c r="C153" s="3" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
@@ -5034,7 +5035,7 @@
         <v>212</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="155" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
@@ -5042,10 +5043,10 @@
         <v>157</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
@@ -5054,7 +5055,7 @@
       </c>
       <c r="B156" s="1"/>
       <c r="C156" s="10" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
@@ -5062,10 +5063,10 @@
         <v>159</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="C157" s="6" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
@@ -5073,484 +5074,482 @@
         <v>160</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="C158" s="3"/>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>462</v>
+        <v>638</v>
       </c>
       <c r="C159" s="3"/>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="C160" s="32" t="s">
-        <v>467</v>
-      </c>
+        <v>461</v>
+      </c>
+      <c r="C160" s="3"/>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B161" s="1"/>
-      <c r="C161" s="3" t="s">
-        <v>464</v>
+        <v>162</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="C161" s="32" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B162" s="1"/>
       <c r="C162" s="3" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B163" s="1"/>
-      <c r="C163" s="10" t="s">
-        <v>469</v>
+      <c r="C163" s="3" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B164" s="1"/>
       <c r="C164" s="10" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="B165" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="C165" s="6" t="s">
-        <v>593</v>
+        <v>166</v>
+      </c>
+      <c r="B165" s="1"/>
+      <c r="C165" s="10" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="B166" s="1"/>
-      <c r="C166" s="3" t="s">
-        <v>471</v>
+        <v>167</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="C166" s="6" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B167" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="C167" s="6" t="s">
-        <v>592</v>
+        <v>168</v>
+      </c>
+      <c r="B167" s="1"/>
+      <c r="C167" s="3" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="C168" s="6" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B168" s="1" t="s">
+      <c r="B169" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C169" s="3"/>
+    </row>
+    <row r="170" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A170" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B170" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="C168" s="3"/>
-    </row>
-    <row r="169" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A169" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="B169" s="1" t="s">
+      <c r="C170" s="31" t="s">
         <v>473</v>
-      </c>
-      <c r="C169" s="31" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A170" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="B170" s="1"/>
-      <c r="C170" s="3" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B171" s="1"/>
       <c r="C171" s="3" t="s">
-        <v>475</v>
+        <v>464</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B172" s="1"/>
       <c r="C172" s="3" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="C173" s="6" t="s">
-        <v>593</v>
+        <v>174</v>
+      </c>
+      <c r="B173" s="1"/>
+      <c r="C173" s="3" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="B174" s="1"/>
-      <c r="C174" s="3" t="s">
-        <v>393</v>
+        <v>175</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="C174" s="6" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B175" s="1"/>
       <c r="C175" s="3" t="s">
-        <v>477</v>
+        <v>392</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B176" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="C176" s="3"/>
+        <v>177</v>
+      </c>
+      <c r="B176" s="1"/>
+      <c r="C176" s="3" t="s">
+        <v>476</v>
+      </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B177" s="1">
-        <v>1</v>
-      </c>
-      <c r="C177" s="3" t="s">
-        <v>479</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="C177" s="3"/>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B178" s="1">
+        <v>1</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B178" s="1" t="s">
-        <v>642</v>
-      </c>
-      <c r="C178" s="3" t="s">
+      <c r="B179" s="1" t="s">
+        <v>629</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B180" s="1"/>
+      <c r="C180" s="10" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A179" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B179" s="1"/>
-      <c r="C179" s="10" t="s">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B181" s="1"/>
+      <c r="C181" s="3" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A180" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B180" s="1"/>
-      <c r="C180" s="3" t="s">
+    <row r="182" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A182" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B182" s="1"/>
+      <c r="C182" s="10" t="s">
         <v>482</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A181" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="B181" s="1"/>
-      <c r="C181" s="10" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A182" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="B182" s="1"/>
-      <c r="C182" s="3" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B183" s="1"/>
       <c r="C183" s="3" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B184" s="1"/>
       <c r="C184" s="3" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B185" s="1"/>
       <c r="C185" s="3" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B186" s="1"/>
       <c r="C186" s="3" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B187" s="1"/>
       <c r="C187" s="3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B188" s="1"/>
       <c r="C188" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B189" s="1"/>
       <c r="C189" s="3" t="s">
-        <v>455</v>
+        <v>488</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B190" s="1"/>
-      <c r="C190" s="10" t="s">
-        <v>490</v>
+      <c r="C190" s="3" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B191" s="1"/>
       <c r="C191" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B192" s="1"/>
       <c r="C192" s="10" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B193" s="1"/>
+      <c r="C193" s="10" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A194" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B194" s="1" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="193" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A193" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B193" s="1" t="s">
+      <c r="C194" s="6" t="s">
         <v>492</v>
-      </c>
-      <c r="C193" s="6" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A194" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="B194" s="1"/>
-      <c r="C194" s="6" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B195" s="1"/>
-      <c r="C195" s="10" t="s">
+      <c r="C195" s="6" t="s">
         <v>495</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B196" s="1"/>
-      <c r="C196" s="3" t="s">
-        <v>497</v>
+      <c r="C196" s="10" t="s">
+        <v>494</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B197" s="1"/>
       <c r="C197" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B198" s="1" t="s">
-        <v>499</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="B198" s="1"/>
       <c r="C198" s="3" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="C200" s="6" t="s">
-        <v>503</v>
+        <v>500</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="B201" s="1">
-        <v>32</v>
-      </c>
-      <c r="C201" s="3" t="s">
-        <v>504</v>
+        <v>202</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="C201" s="6" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="B202" s="1"/>
-      <c r="C202" s="10" t="s">
-        <v>505</v>
+        <v>203</v>
+      </c>
+      <c r="B202" s="1">
+        <v>32</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B203" s="1"/>
+      <c r="C203" s="10" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="B203" s="1"/>
-      <c r="C203" s="3" t="s">
+      <c r="B204" s="1"/>
+      <c r="C204" s="3" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A205" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B205" s="1"/>
+      <c r="C205" s="10" t="s">
         <v>506</v>
-      </c>
-    </row>
-    <row r="204" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A204" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="B204" s="1"/>
-      <c r="C204" s="10" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A205" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="B205" s="1"/>
-      <c r="C205" s="3" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B206" s="1"/>
       <c r="C206" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B207" s="1"/>
+      <c r="C207" s="3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A208" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="B207" s="1"/>
-      <c r="C207" s="6" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="208" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A208" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="B208" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="C208" s="3" t="s">
-        <v>511</v>
+      <c r="B208" s="1"/>
+      <c r="C208" s="6" t="s">
+        <v>509</v>
       </c>
     </row>
     <row r="209" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
@@ -5558,89 +5557,100 @@
         <v>213</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="C209" s="3"/>
+        <v>639</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>510</v>
+      </c>
     </row>
     <row r="210" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>213</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="C210" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="C210" s="3"/>
+    </row>
+    <row r="211" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A211" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B211" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="C211" s="10" t="s">
         <v>214</v>
-      </c>
-    </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A211" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="B211" s="1"/>
-      <c r="C211" s="6" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B212" s="1"/>
+      <c r="C212" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A213" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B213" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="B212" s="1" t="s">
-        <v>515</v>
-      </c>
-      <c r="C212" s="3" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="213" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A213" s="1" t="s">
-        <v>514</v>
-      </c>
-      <c r="B213" s="1" t="s">
+      <c r="C213" s="3" t="s">
         <v>516</v>
-      </c>
-      <c r="C213" s="3" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="214" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
-        <v>226</v>
+        <v>513</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>526</v>
+        <v>515</v>
       </c>
       <c r="C214" s="3" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A215" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B215" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A216" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B216" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="C216" s="3" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A215" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="B215" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="C215" s="3" t="s">
+    <row r="217" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A217" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B217" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="C217" s="3" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A216" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="B216" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="C216" s="3" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A217" s="1"/>
-      <c r="B217" s="1"/>
-      <c r="C217" s="3"/>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A218" s="1"/>
+      <c r="B218" s="1"/>
+      <c r="C218" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5674,101 +5684,101 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
       <c r="B2" s="17"/>
       <c r="C2" s="16" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>529</v>
+        <v>523</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>530</v>
+        <v>524</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="16" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>536</v>
+        <v>530</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -5777,7 +5787,7 @@
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="34" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -5786,7 +5796,7 @@
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -5794,10 +5804,10 @@
         <v>23</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -5808,18 +5818,18 @@
         <v>210</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="B17" s="17">
         <v>0</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -5828,43 +5838,43 @@
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>540</v>
-      </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="34" t="s">
-        <v>586</v>
-      </c>
+        <v>534</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>636</v>
+      </c>
+      <c r="C20" s="34"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="C21" s="17"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="63" x14ac:dyDescent="0.25">
@@ -5872,50 +5882,50 @@
         <v>41</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>588</v>
+        <v>581</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>589</v>
+        <v>582</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="C25" s="34" t="s">
-        <v>594</v>
+        <v>587</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="34" t="s">
-        <v>595</v>
+        <v>588</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="34" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -5924,15 +5934,15 @@
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="C29" s="17"/>
     </row>
@@ -5942,16 +5952,16 @@
       </c>
       <c r="B30" s="17"/>
       <c r="C30" s="17" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="34" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -5960,25 +5970,25 @@
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="17" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="17" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="17" t="s">
-        <v>598</v>
+        <v>591</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="B34" s="17"/>
       <c r="C34" s="17" t="s">
-        <v>599</v>
+        <v>592</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -5987,7 +5997,7 @@
       </c>
       <c r="B35" s="17"/>
       <c r="C35" s="17" t="s">
-        <v>600</v>
+        <v>593</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -5996,84 +6006,84 @@
       </c>
       <c r="B36" s="17"/>
       <c r="C36" s="34" t="s">
-        <v>601</v>
+        <v>594</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>603</v>
+        <v>596</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="17" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>604</v>
+        <v>597</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="17" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>606</v>
+        <v>599</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>605</v>
+        <v>598</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="17" t="s">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
-        <v>556</v>
+        <v>550</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="B43" s="17" t="s">
+        <v>595</v>
+      </c>
+      <c r="C43" s="17" t="s">
         <v>602</v>
-      </c>
-      <c r="C43" s="17" t="s">
-        <v>609</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -6081,83 +6091,83 @@
         <v>180</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>642</v>
+        <v>629</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>610</v>
+        <v>603</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
-        <v>558</v>
-      </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="34" t="s">
-        <v>611</v>
-      </c>
+        <v>552</v>
+      </c>
+      <c r="B45" s="17" t="s">
+        <v>636</v>
+      </c>
+      <c r="C45" s="34"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="C46" s="17"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>612</v>
+        <v>604</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="B48" s="17"/>
       <c r="C48" s="37" t="s">
-        <v>632</v>
+        <v>620</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C49" s="18"/>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="17" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="B50" s="17"/>
       <c r="C50" s="17" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="17" t="s">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>614</v>
+        <v>606</v>
       </c>
       <c r="C51" s="17"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="17" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>642</v>
+        <v>629</v>
       </c>
       <c r="C52" s="17"/>
     </row>
@@ -6167,18 +6177,18 @@
       </c>
       <c r="B53" s="17"/>
       <c r="C53" s="17" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="17" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -6186,10 +6196,10 @@
         <v>202</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
   </sheetData>
@@ -6223,72 +6233,72 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>240</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>243</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>643</v>
+        <v>630</v>
       </c>
       <c r="C5" s="18"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>644</v>
+        <v>631</v>
       </c>
       <c r="C6" s="18"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>633</v>
+        <v>621</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>252</v>
-      </c>
       <c r="C8" s="17" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -6322,150 +6332,150 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B5" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="C5" s="17" t="s">
         <v>331</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B6" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>331</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B7" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>331</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>629</v>
+        <v>617</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
   </sheetData>
@@ -6499,87 +6509,87 @@
     </row>
     <row r="2" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>617</v>
+        <v>609</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>618</v>
+        <v>610</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B5" s="23"/>
       <c r="C5" s="23" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="22" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B7" s="25"/>
       <c r="C7" s="23" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B8" s="25"/>
       <c r="C8" s="25" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B9" s="25"/>
       <c r="C9" s="25" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B10" s="25"/>
       <c r="C10" s="25" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -6588,18 +6598,18 @@
       </c>
       <c r="B11" s="25"/>
       <c r="C11" s="25" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B12" s="28" t="s">
+        <v>357</v>
+      </c>
+      <c r="C12" s="29" t="s">
         <v>358</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -6633,13 +6643,13 @@
     </row>
     <row r="2" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>636</v>
+        <v>623</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>637</v>
+        <v>624</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>638</v>
+        <v>625</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6676,45 +6686,45 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C2" t="s">
-        <v>616</v>
+        <v>608</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
   </sheetData>
@@ -6751,7 +6761,7 @@
         <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6759,7 +6769,7 @@
         <v>174</v>
       </c>
       <c r="C3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Specify key file for ssh into VMs SSH configurations on local side for SSH into VMs Fixed some values in slurm.conf Fix on kickstart as well, with the new ssh configurations
</commit_message>
<xml_diff>
--- a/roles/setup_slurm/files/slurm_conf.xlsx
+++ b/roles/setup_slurm/files/slurm_conf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jsequeira\vs_projects\ansible-puli\roles\setup_slurm\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F413F33-2D18-43BC-B7B0-59C831350A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF14DA18-99E8-4A9D-BCA7-46745C962C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{787EF645-FDEF-D749-B29A-8997BAA1BD7D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{787EF645-FDEF-D749-B29A-8997BAA1BD7D}"/>
   </bookViews>
   <sheets>
     <sheet name="code" sheetId="4" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="slurmdbd.conf" sheetId="15" r:id="rId3"/>
     <sheet name="acct_gather.conf" sheetId="3" r:id="rId4"/>
     <sheet name="cgroup.conf" sheetId="5" r:id="rId5"/>
-    <sheet name="job_container.conf" sheetId="6" r:id="rId6"/>
+    <sheet name="x job_container.conf" sheetId="6" r:id="rId6"/>
     <sheet name="topology.conf" sheetId="19" r:id="rId7"/>
     <sheet name="x helpers.conf" sheetId="7" r:id="rId8"/>
     <sheet name="x nss_slurm.conf" sheetId="9" r:id="rId9"/>
@@ -2173,24 +2173,12 @@
     <t>SwitchName</t>
   </si>
   <si>
-    <t>switch_1 Nodes=cpu[01-11],mem02,gpu[01-02]</t>
-  </si>
-  <si>
     <t>For only consider only one switch, since all servers are connected, in a trunk, to the main switch.</t>
   </si>
   <si>
     <t>{{ sms_name }}</t>
   </si>
   <si>
-    <t>{{ accounting_storage_user }}</t>
-  </si>
-  <si>
-    <t>{{ cluster_name }}</t>
-  </si>
-  <si>
-    <t>{{ slurm_user }}</t>
-  </si>
-  <si>
     <t>{{ bmc_username }}</t>
   </si>
   <si>
@@ -2234,6 +2222,18 @@
   </si>
   <si>
     <t>gpu Nodes=scc-gpu[01-02]-10G MaxTime=10-00:00:00 AllowAccounts=GPU AllowGroups=LAMSA CpuBind=core DefMemPerCPU=5333</t>
+  </si>
+  <si>
+    <t>{{ setup_slurm_accounting_storage_user }}</t>
+  </si>
+  <si>
+    <t>{{ setup_slurm_cluster_name }}</t>
+  </si>
+  <si>
+    <t>{{ setup_slurm_slurm_user }}</t>
+  </si>
+  <si>
+    <t>switch_1 Nodes=scc-cpu[01-11]-10G,scc-mem[01-02]-10G,scc-gpu[01-02]-10G</t>
   </si>
 </sst>
 </file>
@@ -3583,7 +3583,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="C2" s="6"/>
     </row>
@@ -3612,7 +3612,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -3674,7 +3674,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>627</v>
+        <v>641</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>612</v>
@@ -3861,7 +3861,7 @@
         <v>32</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>628</v>
+        <v>642</v>
       </c>
       <c r="C30" s="6"/>
     </row>
@@ -4029,7 +4029,7 @@
         <v>613</v>
       </c>
       <c r="C48" s="36" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -4164,7 +4164,7 @@
         <v>64</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>614</v>
@@ -4224,7 +4224,7 @@
         <v>70</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C68" s="3"/>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="B131" s="1"/>
       <c r="C131" s="38" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -5074,7 +5074,7 @@
         <v>160</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="C158" s="3"/>
     </row>
@@ -5083,7 +5083,7 @@
         <v>160</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="C159" s="3"/>
     </row>
@@ -5275,7 +5275,7 @@
         <v>180</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>629</v>
+        <v>643</v>
       </c>
       <c r="C179" s="3" t="s">
         <v>479</v>
@@ -5557,7 +5557,7 @@
         <v>213</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="C209" s="3" t="s">
         <v>510</v>
@@ -5568,7 +5568,7 @@
         <v>213</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="C210" s="3"/>
     </row>
@@ -5577,7 +5577,7 @@
         <v>213</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="C211" s="10" t="s">
         <v>214</v>
@@ -5619,7 +5619,7 @@
         <v>225</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="C215" s="3" t="s">
         <v>517</v>
@@ -5630,7 +5630,7 @@
         <v>225</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="C216" s="3" t="s">
         <v>518</v>
@@ -5641,7 +5641,7 @@
         <v>225</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="C217" s="3" t="s">
         <v>519</v>
@@ -5855,7 +5855,7 @@
         <v>534</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="C20" s="34"/>
     </row>
@@ -5864,7 +5864,7 @@
         <v>535</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="C21" s="17"/>
     </row>
@@ -6091,7 +6091,7 @@
         <v>180</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>629</v>
+        <v>643</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>603</v>
@@ -6102,7 +6102,7 @@
         <v>552</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="C45" s="34"/>
     </row>
@@ -6111,7 +6111,7 @@
         <v>553</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="C46" s="17"/>
     </row>
@@ -6167,7 +6167,7 @@
         <v>559</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>629</v>
+        <v>643</v>
       </c>
       <c r="C52" s="17"/>
     </row>
@@ -6266,7 +6266,7 @@
         <v>244</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C5" s="18"/>
     </row>
@@ -6275,7 +6275,7 @@
         <v>245</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="C6" s="18"/>
     </row>
@@ -6646,10 +6646,10 @@
         <v>623</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="C2" s="37" t="s">
         <v>624</v>
-      </c>
-      <c r="C2" s="37" t="s">
-        <v>625</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Proper hosts file for ssh connection Added encrypted munge key, because ansible can't read from /etc/munge Fix in "sms" vs "master_hostname" Added DNS resolution to kickstart of VMs SSH configuration now allows for root ssh through hostname
</commit_message>
<xml_diff>
--- a/roles/setup_slurm/files/slurm_conf.xlsx
+++ b/roles/setup_slurm/files/slurm_conf.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jsequeira\vs_projects\ansible-puli\roles\setup_slurm\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF14DA18-99E8-4A9D-BCA7-46745C962C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD25E764-D235-4CA8-BFF1-B6EED89FB3BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{787EF645-FDEF-D749-B29A-8997BAA1BD7D}"/>
   </bookViews>
@@ -2176,9 +2176,6 @@
     <t>For only consider only one switch, since all servers are connected, in a trunk, to the main switch.</t>
   </si>
   <si>
-    <t>{{ sms_name }}</t>
-  </si>
-  <si>
     <t>{{ bmc_username }}</t>
   </si>
   <si>
@@ -2234,6 +2231,9 @@
   </si>
   <si>
     <t>switch_1 Nodes=scc-cpu[01-11]-10G,scc-mem[01-02]-10G,scc-gpu[01-02]-10G</t>
+  </si>
+  <si>
+    <t>Redundant if using the database</t>
   </si>
 </sst>
 </file>
@@ -3583,7 +3583,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C2" s="6"/>
     </row>
@@ -3612,7 +3612,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -3674,7 +3674,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>612</v>
@@ -3861,7 +3861,7 @@
         <v>32</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="C30" s="6"/>
     </row>
@@ -4029,7 +4029,7 @@
         <v>613</v>
       </c>
       <c r="C48" s="36" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -4164,7 +4164,7 @@
         <v>64</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>614</v>
@@ -4223,10 +4223,10 @@
       <c r="A68" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>625</v>
-      </c>
-      <c r="C68" s="3"/>
+      <c r="B68" s="1"/>
+      <c r="C68" s="3" t="s">
+        <v>644</v>
+      </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="B131" s="1"/>
       <c r="C131" s="38" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -5074,7 +5074,7 @@
         <v>160</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C158" s="3"/>
     </row>
@@ -5083,7 +5083,7 @@
         <v>160</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="C159" s="3"/>
     </row>
@@ -5275,7 +5275,7 @@
         <v>180</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C179" s="3" t="s">
         <v>479</v>
@@ -5557,7 +5557,7 @@
         <v>213</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C209" s="3" t="s">
         <v>510</v>
@@ -5568,7 +5568,7 @@
         <v>213</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="C210" s="3"/>
     </row>
@@ -5577,7 +5577,7 @@
         <v>213</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C211" s="10" t="s">
         <v>214</v>
@@ -5619,7 +5619,7 @@
         <v>225</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C215" s="3" t="s">
         <v>517</v>
@@ -5630,7 +5630,7 @@
         <v>225</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C216" s="3" t="s">
         <v>518</v>
@@ -5641,7 +5641,7 @@
         <v>225</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="C217" s="3" t="s">
         <v>519</v>
@@ -5855,7 +5855,7 @@
         <v>534</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C20" s="34"/>
     </row>
@@ -5864,7 +5864,7 @@
         <v>535</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C21" s="17"/>
     </row>
@@ -6091,7 +6091,7 @@
         <v>180</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>603</v>
@@ -6102,7 +6102,7 @@
         <v>552</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C45" s="34"/>
     </row>
@@ -6111,7 +6111,7 @@
         <v>553</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C46" s="17"/>
     </row>
@@ -6167,7 +6167,7 @@
         <v>559</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C52" s="17"/>
     </row>
@@ -6266,7 +6266,7 @@
         <v>244</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C5" s="18"/>
     </row>
@@ -6275,7 +6275,7 @@
         <v>245</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C6" s="18"/>
     </row>
@@ -6646,7 +6646,7 @@
         <v>623</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C2" s="37" t="s">
         <v>624</v>

</xml_diff>